<commit_message>
Add switchable project currency
</commit_message>
<xml_diff>
--- a/starter/ledger_starter_workbook.xlsx
+++ b/starter/ledger_starter_workbook.xlsx
@@ -655,6 +655,90 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>CAD</t>
+        </is>
+      </c>
+      <c r="B8">
+        <v>0.6700</v>
+      </c>
+      <c r="C8">
+        <v>0.7280</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>starter</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Offline starter rate</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>AUD</t>
+        </is>
+      </c>
+      <c r="B9">
+        <v>0.6100</v>
+      </c>
+      <c r="C9">
+        <v>0.6630</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>starter</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Offline starter rate</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>JPY</t>
+        </is>
+      </c>
+      <c r="B10">
+        <v>0.0060</v>
+      </c>
+      <c r="C10">
+        <v>0.0065</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>starter</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Offline starter rate</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -1056,7 +1140,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -1170,7 +1254,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -1284,7 +1368,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -1398,7 +1482,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -1512,7 +1596,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -1626,7 +1710,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -1740,7 +1824,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -1854,7 +1938,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -1968,7 +2052,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -2082,7 +2166,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -2196,7 +2280,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -2310,7 +2394,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -2424,7 +2508,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -2538,7 +2622,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -2652,7 +2736,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -2766,7 +2850,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -2880,7 +2964,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -2994,7 +3078,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -3108,7 +3192,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -3222,7 +3306,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -3336,7 +3420,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -3450,7 +3534,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -3564,7 +3648,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -3678,7 +3762,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -3792,7 +3876,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
@@ -3906,7 +3990,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -4020,7 +4104,7 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -4134,7 +4218,7 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
@@ -4248,7 +4332,7 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -4362,7 +4446,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -4476,7 +4560,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -4590,7 +4674,7 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -4704,7 +4788,7 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
@@ -4818,7 +4902,7 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -4932,7 +5016,7 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
@@ -5046,7 +5130,7 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
@@ -5160,7 +5244,7 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
@@ -5274,7 +5358,7 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
@@ -5388,7 +5472,7 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
@@ -5502,7 +5586,7 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
@@ -5616,7 +5700,7 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
@@ -5730,7 +5814,7 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
@@ -5844,7 +5928,7 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
@@ -5958,7 +6042,7 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
@@ -6072,7 +6156,7 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
@@ -6186,7 +6270,7 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
@@ -6300,7 +6384,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
@@ -6414,7 +6498,7 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
@@ -6528,7 +6612,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -6642,7 +6726,7 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -6756,7 +6840,7 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
@@ -6870,7 +6954,7 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
@@ -6984,7 +7068,7 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
@@ -7098,7 +7182,7 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
@@ -7212,7 +7296,7 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
@@ -7326,7 +7410,7 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
@@ -7440,7 +7524,7 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
@@ -7554,7 +7638,7 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
@@ -7668,7 +7752,7 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
@@ -7782,7 +7866,7 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
@@ -7896,7 +7980,7 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
@@ -8010,7 +8094,7 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
@@ -8124,7 +8208,7 @@
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
@@ -8238,7 +8322,7 @@
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
@@ -8352,7 +8436,7 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
@@ -8466,7 +8550,7 @@
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
@@ -8580,7 +8664,7 @@
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
@@ -8694,7 +8778,7 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
@@ -8808,7 +8892,7 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
@@ -8922,7 +9006,7 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J71" t="inlineStr">
@@ -9036,7 +9120,7 @@
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
@@ -9150,7 +9234,7 @@
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
@@ -9264,7 +9348,7 @@
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J74" t="inlineStr">
@@ -9378,7 +9462,7 @@
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J75" t="inlineStr">
@@ -9492,7 +9576,7 @@
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J76" t="inlineStr">
@@ -9606,7 +9690,7 @@
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
@@ -9720,7 +9804,7 @@
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J78" t="inlineStr">
@@ -9834,7 +9918,7 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
@@ -9948,7 +10032,7 @@
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J80" t="inlineStr">
@@ -10062,7 +10146,7 @@
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
@@ -10176,7 +10260,7 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J82" t="inlineStr">
@@ -10290,7 +10374,7 @@
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
@@ -10404,7 +10488,7 @@
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J84" t="inlineStr">
@@ -10518,7 +10602,7 @@
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J85" t="inlineStr">
@@ -10632,7 +10716,7 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J86" t="inlineStr">
@@ -10746,7 +10830,7 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
@@ -10860,7 +10944,7 @@
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J88" t="inlineStr">
@@ -10974,7 +11058,7 @@
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
@@ -11088,7 +11172,7 @@
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J90" t="inlineStr">
@@ -11202,7 +11286,7 @@
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J91" t="inlineStr">
@@ -11316,7 +11400,7 @@
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J92" t="inlineStr">
@@ -11430,7 +11514,7 @@
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J93" t="inlineStr">
@@ -11544,7 +11628,7 @@
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J94" t="inlineStr">
@@ -11658,7 +11742,7 @@
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J95" t="inlineStr">
@@ -11772,7 +11856,7 @@
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J96" t="inlineStr">
@@ -11886,7 +11970,7 @@
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J97" t="inlineStr">
@@ -12000,7 +12084,7 @@
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J98" t="inlineStr">
@@ -12114,7 +12198,7 @@
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J99" t="inlineStr">
@@ -12228,7 +12312,7 @@
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J100" t="inlineStr">
@@ -12342,7 +12426,7 @@
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J101" t="inlineStr">
@@ -12456,7 +12540,7 @@
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J102" t="inlineStr">
@@ -12570,7 +12654,7 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
@@ -12684,7 +12768,7 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J104" t="inlineStr">
@@ -12798,7 +12882,7 @@
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J105" t="inlineStr">
@@ -12912,7 +12996,7 @@
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J106" t="inlineStr">
@@ -13026,7 +13110,7 @@
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J107" t="inlineStr">
@@ -13140,7 +13224,7 @@
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J108" t="inlineStr">
@@ -13254,7 +13338,7 @@
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J109" t="inlineStr">
@@ -13368,7 +13452,7 @@
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J110" t="inlineStr">
@@ -13482,7 +13566,7 @@
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J111" t="inlineStr">
@@ -13596,7 +13680,7 @@
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J112" t="inlineStr">
@@ -13710,7 +13794,7 @@
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J113" t="inlineStr">
@@ -13824,7 +13908,7 @@
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J114" t="inlineStr">
@@ -13938,7 +14022,7 @@
       </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J115" t="inlineStr">
@@ -14052,7 +14136,7 @@
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J116" t="inlineStr">
@@ -14166,7 +14250,7 @@
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J117" t="inlineStr">
@@ -14280,7 +14364,7 @@
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J118" t="inlineStr">
@@ -14394,7 +14478,7 @@
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J119" t="inlineStr">
@@ -14508,7 +14592,7 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J120" t="inlineStr">
@@ -14622,7 +14706,7 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J121" t="inlineStr">
@@ -14736,7 +14820,7 @@
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J122" t="inlineStr">
@@ -14850,7 +14934,7 @@
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J123" t="inlineStr">
@@ -14964,7 +15048,7 @@
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J124" t="inlineStr">
@@ -15078,7 +15162,7 @@
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J125" t="inlineStr">
@@ -15192,7 +15276,7 @@
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J126" t="inlineStr">
@@ -15306,7 +15390,7 @@
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J127" t="inlineStr">
@@ -15420,7 +15504,7 @@
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J128" t="inlineStr">
@@ -15534,7 +15618,7 @@
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J129" t="inlineStr">
@@ -15648,7 +15732,7 @@
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J130" t="inlineStr">
@@ -15762,7 +15846,7 @@
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
@@ -15876,7 +15960,7 @@
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J132" t="inlineStr">
@@ -15990,7 +16074,7 @@
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J133" t="inlineStr">
@@ -16104,7 +16188,7 @@
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J134" t="inlineStr">
@@ -16218,7 +16302,7 @@
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J135" t="inlineStr">
@@ -16332,7 +16416,7 @@
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J136" t="inlineStr">
@@ -16446,7 +16530,7 @@
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J137" t="inlineStr">
@@ -16560,7 +16644,7 @@
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J138" t="inlineStr">
@@ -16674,7 +16758,7 @@
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J139" t="inlineStr">
@@ -16788,7 +16872,7 @@
       </c>
       <c r="I140" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J140" t="inlineStr">
@@ -16902,7 +16986,7 @@
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J141" t="inlineStr">
@@ -17016,7 +17100,7 @@
       </c>
       <c r="I142" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J142" t="inlineStr">
@@ -17130,7 +17214,7 @@
       </c>
       <c r="I143" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J143" t="inlineStr">
@@ -17244,7 +17328,7 @@
       </c>
       <c r="I144" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J144" t="inlineStr">
@@ -17358,7 +17442,7 @@
       </c>
       <c r="I145" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J145" t="inlineStr">
@@ -17472,7 +17556,7 @@
       </c>
       <c r="I146" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J146" t="inlineStr">
@@ -17586,7 +17670,7 @@
       </c>
       <c r="I147" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J147" t="inlineStr">
@@ -17700,7 +17784,7 @@
       </c>
       <c r="I148" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J148" t="inlineStr">
@@ -17814,7 +17898,7 @@
       </c>
       <c r="I149" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J149" t="inlineStr">
@@ -17928,7 +18012,7 @@
       </c>
       <c r="I150" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J150" t="inlineStr">
@@ -18042,7 +18126,7 @@
       </c>
       <c r="I151" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J151" t="inlineStr">
@@ -18156,7 +18240,7 @@
       </c>
       <c r="I152" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J152" t="inlineStr">
@@ -18270,7 +18354,7 @@
       </c>
       <c r="I153" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J153" t="inlineStr">
@@ -18384,7 +18468,7 @@
       </c>
       <c r="I154" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J154" t="inlineStr">
@@ -18498,7 +18582,7 @@
       </c>
       <c r="I155" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J155" t="inlineStr">
@@ -18612,7 +18696,7 @@
       </c>
       <c r="I156" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J156" t="inlineStr">
@@ -18726,7 +18810,7 @@
       </c>
       <c r="I157" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J157" t="inlineStr">
@@ -18840,7 +18924,7 @@
       </c>
       <c r="I158" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J158" t="inlineStr">
@@ -18954,7 +19038,7 @@
       </c>
       <c r="I159" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J159" t="inlineStr">
@@ -19068,7 +19152,7 @@
       </c>
       <c r="I160" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J160" t="inlineStr">
@@ -19182,7 +19266,7 @@
       </c>
       <c r="I161" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J161" t="inlineStr">
@@ -19296,7 +19380,7 @@
       </c>
       <c r="I162" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J162" t="inlineStr">
@@ -19410,7 +19494,7 @@
       </c>
       <c r="I163" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J163" t="inlineStr">
@@ -19524,7 +19608,7 @@
       </c>
       <c r="I164" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J164" t="inlineStr">
@@ -19638,7 +19722,7 @@
       </c>
       <c r="I165" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J165" t="inlineStr">
@@ -19752,7 +19836,7 @@
       </c>
       <c r="I166" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J166" t="inlineStr">
@@ -19866,7 +19950,7 @@
       </c>
       <c r="I167" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J167" t="inlineStr">
@@ -19980,7 +20064,7 @@
       </c>
       <c r="I168" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J168" t="inlineStr">
@@ -20094,7 +20178,7 @@
       </c>
       <c r="I169" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J169" t="inlineStr">
@@ -20208,7 +20292,7 @@
       </c>
       <c r="I170" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J170" t="inlineStr">
@@ -20322,7 +20406,7 @@
       </c>
       <c r="I171" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J171" t="inlineStr">
@@ -20436,7 +20520,7 @@
       </c>
       <c r="I172" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J172" t="inlineStr">
@@ -20550,7 +20634,7 @@
       </c>
       <c r="I173" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J173" t="inlineStr">
@@ -20664,7 +20748,7 @@
       </c>
       <c r="I174" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J174" t="inlineStr">
@@ -20778,7 +20862,7 @@
       </c>
       <c r="I175" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J175" t="inlineStr">
@@ -20892,7 +20976,7 @@
       </c>
       <c r="I176" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J176" t="inlineStr">
@@ -21006,7 +21090,7 @@
       </c>
       <c r="I177" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J177" t="inlineStr">
@@ -21120,7 +21204,7 @@
       </c>
       <c r="I178" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J178" t="inlineStr">
@@ -21234,7 +21318,7 @@
       </c>
       <c r="I179" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J179" t="inlineStr">
@@ -21348,7 +21432,7 @@
       </c>
       <c r="I180" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J180" t="inlineStr">
@@ -21462,7 +21546,7 @@
       </c>
       <c r="I181" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J181" t="inlineStr">
@@ -21576,7 +21660,7 @@
       </c>
       <c r="I182" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J182" t="inlineStr">
@@ -21690,7 +21774,7 @@
       </c>
       <c r="I183" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J183" t="inlineStr">
@@ -21804,7 +21888,7 @@
       </c>
       <c r="I184" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J184" t="inlineStr">
@@ -21918,7 +22002,7 @@
       </c>
       <c r="I185" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J185" t="inlineStr">
@@ -22032,7 +22116,7 @@
       </c>
       <c r="I186" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J186" t="inlineStr">
@@ -22146,7 +22230,7 @@
       </c>
       <c r="I187" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J187" t="inlineStr">
@@ -22260,7 +22344,7 @@
       </c>
       <c r="I188" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J188" t="inlineStr">
@@ -22374,7 +22458,7 @@
       </c>
       <c r="I189" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J189" t="inlineStr">
@@ -22488,7 +22572,7 @@
       </c>
       <c r="I190" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J190" t="inlineStr">
@@ -22602,7 +22686,7 @@
       </c>
       <c r="I191" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J191" t="inlineStr">
@@ -22716,7 +22800,7 @@
       </c>
       <c r="I192" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J192" t="inlineStr">
@@ -22830,7 +22914,7 @@
       </c>
       <c r="I193" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J193" t="inlineStr">
@@ -22944,7 +23028,7 @@
       </c>
       <c r="I194" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J194" t="inlineStr">
@@ -23058,7 +23142,7 @@
       </c>
       <c r="I195" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J195" t="inlineStr">
@@ -23172,7 +23256,7 @@
       </c>
       <c r="I196" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J196" t="inlineStr">
@@ -23286,7 +23370,7 @@
       </c>
       <c r="I197" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J197" t="inlineStr">
@@ -23400,7 +23484,7 @@
       </c>
       <c r="I198" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J198" t="inlineStr">
@@ -23514,7 +23598,7 @@
       </c>
       <c r="I199" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J199" t="inlineStr">
@@ -23628,7 +23712,7 @@
       </c>
       <c r="I200" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J200" t="inlineStr">
@@ -23742,7 +23826,7 @@
       </c>
       <c r="I201" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J201" t="inlineStr">
@@ -23856,7 +23940,7 @@
       </c>
       <c r="I202" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J202" t="inlineStr">
@@ -23970,7 +24054,7 @@
       </c>
       <c r="I203" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J203" t="inlineStr">
@@ -24084,7 +24168,7 @@
       </c>
       <c r="I204" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J204" t="inlineStr">
@@ -24198,7 +24282,7 @@
       </c>
       <c r="I205" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J205" t="inlineStr">
@@ -24312,7 +24396,7 @@
       </c>
       <c r="I206" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J206" t="inlineStr">
@@ -24426,7 +24510,7 @@
       </c>
       <c r="I207" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J207" t="inlineStr">
@@ -24540,7 +24624,7 @@
       </c>
       <c r="I208" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J208" t="inlineStr">
@@ -24654,7 +24738,7 @@
       </c>
       <c r="I209" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J209" t="inlineStr">
@@ -24768,7 +24852,7 @@
       </c>
       <c r="I210" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J210" t="inlineStr">
@@ -24882,7 +24966,7 @@
       </c>
       <c r="I211" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J211" t="inlineStr">
@@ -24996,7 +25080,7 @@
       </c>
       <c r="I212" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J212" t="inlineStr">
@@ -25110,7 +25194,7 @@
       </c>
       <c r="I213" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J213" t="inlineStr">
@@ -25224,7 +25308,7 @@
       </c>
       <c r="I214" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J214" t="inlineStr">
@@ -25338,7 +25422,7 @@
       </c>
       <c r="I215" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J215" t="inlineStr">
@@ -25452,7 +25536,7 @@
       </c>
       <c r="I216" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J216" t="inlineStr">
@@ -25566,7 +25650,7 @@
       </c>
       <c r="I217" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J217" t="inlineStr">
@@ -25680,7 +25764,7 @@
       </c>
       <c r="I218" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J218" t="inlineStr">
@@ -25794,7 +25878,7 @@
       </c>
       <c r="I219" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J219" t="inlineStr">
@@ -25908,7 +25992,7 @@
       </c>
       <c r="I220" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J220" t="inlineStr">
@@ -26022,7 +26106,7 @@
       </c>
       <c r="I221" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J221" t="inlineStr">
@@ -26136,7 +26220,7 @@
       </c>
       <c r="I222" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J222" t="inlineStr">
@@ -26250,7 +26334,7 @@
       </c>
       <c r="I223" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J223" t="inlineStr">
@@ -26364,7 +26448,7 @@
       </c>
       <c r="I224" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J224" t="inlineStr">
@@ -26478,7 +26562,7 @@
       </c>
       <c r="I225" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J225" t="inlineStr">
@@ -26592,7 +26676,7 @@
       </c>
       <c r="I226" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J226" t="inlineStr">
@@ -26706,7 +26790,7 @@
       </c>
       <c r="I227" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J227" t="inlineStr">
@@ -26820,7 +26904,7 @@
       </c>
       <c r="I228" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J228" t="inlineStr">
@@ -26934,7 +27018,7 @@
       </c>
       <c r="I229" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J229" t="inlineStr">
@@ -27048,7 +27132,7 @@
       </c>
       <c r="I230" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J230" t="inlineStr">
@@ -27162,7 +27246,7 @@
       </c>
       <c r="I231" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J231" t="inlineStr">
@@ -27276,7 +27360,7 @@
       </c>
       <c r="I232" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J232" t="inlineStr">
@@ -27390,7 +27474,7 @@
       </c>
       <c r="I233" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J233" t="inlineStr">
@@ -27504,7 +27588,7 @@
       </c>
       <c r="I234" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J234" t="inlineStr">
@@ -27618,7 +27702,7 @@
       </c>
       <c r="I235" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J235" t="inlineStr">
@@ -27732,7 +27816,7 @@
       </c>
       <c r="I236" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J236" t="inlineStr">
@@ -27846,7 +27930,7 @@
       </c>
       <c r="I237" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J237" t="inlineStr">
@@ -27960,7 +28044,7 @@
       </c>
       <c r="I238" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J238" t="inlineStr">
@@ -28074,7 +28158,7 @@
       </c>
       <c r="I239" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J239" t="inlineStr">
@@ -28188,7 +28272,7 @@
       </c>
       <c r="I240" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J240" t="inlineStr">
@@ -28302,7 +28386,7 @@
       </c>
       <c r="I241" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J241" t="inlineStr">
@@ -28416,7 +28500,7 @@
       </c>
       <c r="I242" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J242" t="inlineStr">
@@ -28530,7 +28614,7 @@
       </c>
       <c r="I243" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J243" t="inlineStr">
@@ -28644,7 +28728,7 @@
       </c>
       <c r="I244" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J244" t="inlineStr">
@@ -28758,7 +28842,7 @@
       </c>
       <c r="I245" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J245" t="inlineStr">
@@ -28872,7 +28956,7 @@
       </c>
       <c r="I246" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J246" t="inlineStr">
@@ -28986,7 +29070,7 @@
       </c>
       <c r="I247" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J247" t="inlineStr">
@@ -29100,7 +29184,7 @@
       </c>
       <c r="I248" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J248" t="inlineStr">
@@ -29214,7 +29298,7 @@
       </c>
       <c r="I249" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J249" t="inlineStr">
@@ -29328,7 +29412,7 @@
       </c>
       <c r="I250" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J250" t="inlineStr">
@@ -29442,7 +29526,7 @@
       </c>
       <c r="I251" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J251" t="inlineStr">
@@ -29556,7 +29640,7 @@
       </c>
       <c r="I252" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J252" t="inlineStr">
@@ -29670,7 +29754,7 @@
       </c>
       <c r="I253" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J253" t="inlineStr">
@@ -29784,7 +29868,7 @@
       </c>
       <c r="I254" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J254" t="inlineStr">
@@ -29898,7 +29982,7 @@
       </c>
       <c r="I255" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J255" t="inlineStr">
@@ -30012,7 +30096,7 @@
       </c>
       <c r="I256" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J256" t="inlineStr">
@@ -30126,7 +30210,7 @@
       </c>
       <c r="I257" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J257" t="inlineStr">
@@ -30240,7 +30324,7 @@
       </c>
       <c r="I258" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J258" t="inlineStr">
@@ -30354,7 +30438,7 @@
       </c>
       <c r="I259" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J259" t="inlineStr">
@@ -30468,7 +30552,7 @@
       </c>
       <c r="I260" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J260" t="inlineStr">
@@ -30582,7 +30666,7 @@
       </c>
       <c r="I261" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J261" t="inlineStr">
@@ -30696,7 +30780,7 @@
       </c>
       <c r="I262" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J262" t="inlineStr">
@@ -30810,7 +30894,7 @@
       </c>
       <c r="I263" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J263" t="inlineStr">
@@ -30924,7 +31008,7 @@
       </c>
       <c r="I264" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J264" t="inlineStr">
@@ -31038,7 +31122,7 @@
       </c>
       <c r="I265" t="inlineStr">
         <is>
-          <t>Local Ledger</t>
+          <t>Ledger Public Starter</t>
         </is>
       </c>
       <c r="J265" t="inlineStr">

</xml_diff>

<commit_message>
Add INR project currency and changelog fallback
</commit_message>
<xml_diff>
--- a/starter/ledger_starter_workbook.xlsx
+++ b/starter/ledger_starter_workbook.xlsx
@@ -714,26 +714,54 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="B10">
+        <v>0.0110</v>
+      </c>
+      <c r="C10">
+        <v>0.0120</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>starter</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Offline starter rate</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>JPY</t>
         </is>
       </c>
-      <c r="B10">
+      <c r="B11">
         <v>0.0060</v>
       </c>
-      <c r="C10">
+      <c r="C11">
         <v>0.0065</v>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>2026-06-10</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>starter</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>Offline starter rate</t>
         </is>

</xml_diff>

<commit_message>
Add account country support
</commit_message>
<xml_diff>
--- a/starter/ledger_starter_workbook.xlsx
+++ b/starter/ledger_starter_workbook.xlsx
@@ -96,6 +96,11 @@
           <t>notes</t>
         </is>
       </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>country_code</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -167,6 +172,11 @@
           <t>Main operating account</t>
         </is>
       </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -238,6 +248,11 @@
           <t>Six-month liquidity reserve</t>
         </is>
       </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -309,6 +324,11 @@
           <t>ETF and equity portfolio held in USD</t>
         </is>
       </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -380,6 +400,11 @@
           <t>Long-term pension capital in local currency</t>
         </is>
       </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -445,6 +470,11 @@
       <c r="O6" t="inlineStr">
         <is>
           <t>Paid monthly</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t/>
         </is>
       </c>
     </row>

</xml_diff>